<commit_message>
Added parallel workflow where resume customization and resolving url run parallelly
</commit_message>
<xml_diff>
--- a/data/applied_jobs.xlsx
+++ b/data/applied_jobs.xlsx
@@ -446,12 +446,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V46"/>
+  <dimension ref="A1:V48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="33.85714285714285" customWidth="1" min="1" max="1"/>
     <col width="42.14285714285715" customWidth="1" min="2" max="2"/>
-    <col width="13.57142857142857" customWidth="1" min="3" max="24"/>
+    <col width="13.57142857142857" customWidth="1" min="3" max="8"/>
+    <col width="39" customWidth="1" min="9" max="9"/>
+    <col width="13.57142857142857" customWidth="1" min="10" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2531,22 +2533,22 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Software Engineering Full-Time Campus Hire - NYC 2027</t>
+          <t>Junior Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Two Sigma</t>
+          <t>OKAYA INFOCOM</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Milford, OH</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>9 hours ago</t>
+          <t>12 hours ago</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2556,52 +2558,39 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>$225K/yr - $225K/yr</t>
+          <t>null</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Two Sigma is a quantitative investment management and trading firm that combines technology, artificial intelligence, data science, and quantitative research. The full-time campus hire will join a general Software Engineering role, building scalable infrastructure, reliable systems, trading technology, data ingestion platforms, and productivity tools across the organization.
-Responsibilities
-- Building the underlying infrastructure that virtually every other engineering team at Two Sigma uses, such as our distributed storage and public and private cloud environments
-- Ensuring the reliability of "mission critical" products and systems vital to Two Sigma, such as our main trading system
-- Using a suite of open source and proprietary tools to build the environments that test and deploy our quantitative strategies, also known as models
-- Building and maintaining the low-latency, high-performance infrastructure and systems responsible for executing trades
-- Building and scaling the infrastructure used to ingest data from 10,000+ sources daily
-- Partnering with our Corporate teams to develop tools, systems and products responsible for increasing productivity and efficiency across the organization
-Qualification
-Required
-- A Bachelor's, Master's, or PhD degree in a technical or quantitative field
-- Experience with Java, C, C++, Python, Ruby, Perl, or other languages that target the JVM
-- Experience in large-scale systems
-- Exceptional programming skills
-- Strong analytical, organizational, and interpersonal skills
-- A passion of building quality software
-- We are open-minded in our search for critical thinkers who are passionate about technology
-- financial experience is not a requirement
-Benefits
-- Fully paid medical and dental insurance premiums for employees and dependents
-- Competitive 401k match
-- Employer-paid life &amp; disability insurance
-- Onsite gyms with laundry service
-- Wellness activities
-- Casual dress
-- Snacks
-- Game rooms
-- Tuition reimbursement
-- Conference and training sponsorship
-- Generous vacation
-- Unlimited sick days
-- Competitive paid caregiver leaves
-- Flexible in-office days with budget for home office setup
-- Discretionary bonus
-- Health, dental and other wellness plans
-- 401(k) contributions</t>
+          <t>Junior Forward Deployed Engineer - Milford, OH (Full-time, Onsite, Entry Level, 1+ years exp)
+Hiring Manager: Mukesh Prasad
+OKAYA INFOCOM is hiring a Junior Forward Deployed Engineer to develop and support technical solutions for customer business challenges. The role focuses on building applications, APIs, integrations, and proofs of concept while applying AI/GenAI, cloud, containerization, and CI/CD technologies and troubleshooting production issues.
+Responsibilities:
+- Understand customer business challenges and translate them into scalable technical solutions
+- Design, develop, test, and deploy applications, APIs, and integrations using modern engineering practices
+- Build Proof of Concepts (PoCs) and rapidly prototype solutions to validate business and technical requirements
+- Continuously evaluate and apply emerging technologies, including AI/GenAI capabilities, to solve enterprise problems
+- Troubleshoot application, integration, and production issues through systematic debugging and root cause analysis
+- Work with Cloud, Containerization, and CI/CD technologies to support production deployments
+Qualifications:
+Python, SQL, Data Processing, Relational Databases, REST APIs, Enterprise Integrations, Data Structures and Algorithms, Git, CI/CD, Cloud Platforms AWS, Cloud Platforms Azure, Cloud Platforms GCP, Docker, Kubernetes, Large Language Models (LLMs), Prompt Engineering, Retrieval-Augmented Generation (RAG), Application Troubleshooting and Testing
+Required:
+· Must have hands-on programming experience in Python with strong coding and debugging skills
+· Must have experience in SQL, data processing, and relational database concepts
+· Must have experience in developing and consuming REST APIs and enterprise integrations
+· Must have strong understanding of Data Structures, Algorithms, and Problem-solving techniques
+· Must have experience with Git, version control, and CI/CD practices
+· Must have working knowledge of Cloud Platforms (AWS, Azure, or GCP) and containerization (Docker/Kubernetes)
+· Must have 1 year experience building or supporting AI/GenAI applications using LLMs, Prompt Engineering, and RAG concepts
+· Must have minimum 1 year experience in application troubleshooting, testing, deployment, and production Support
+Company:
+OKAYA INFOCOM - IT staffing, talent acquisition, and technology solutions partner. Founded in 2006, Holbrook, New York, USA, 201-500 employees. https://www.okayainfo.com</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>New Grad</t>
+          <t>Entry Level</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2616,7 +2605,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>2026-09-09 00:47:28</t>
+          <t>2026-09-09 06:50:53</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2626,7 +2615,7 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>Gmail from Two Sigma Recruiting confirms successfully received application for Software Engineering Full-Time Campus Hire (NYC).</t>
+          <t>Confirmation email from jobs@janestreet.com with subject 'Thank you for applying to Jane Street' explicitly confirms receipt: 'confirm that we received your resume' for Jane Street.</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -4608,6 +4597,186 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>url:3025b0ba356efc6a731c</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Software Engineer - New Grad</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Scale AI</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2 days ago</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/jobs/info/6a9af73bd5ff1f3f1c39caae</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>$124K/yr - $162K/yr</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Scale AI develops reliable AI systems, data, and full-stack technologies that support leading models and enterprise and government applications. The New Grad Software Engineer will own customer-facing product engineering work, shipping and iterating on AI products, data systems, applications, and infrastructure at scale.
+Responsibilities:
+- Build reinforcement learning and post-training data pipelines that power frontier model development
+- Develop evaluation infrastructure that measures model reliability for enterprise and public sector customers
+- Ship agentic AI applications and the tooling that makes them observable, testable, and safe to deploy
+- Ship tools that accelerate the growth of new qualified contributors on Scale's platform
+- Build fraud-detection systems that remove bad actors and keep Scale's contributor base safe and trusted
+- Use models to estimate the quality of tasks and contributors, and guarantee quality on requests at large scale
+- Devise advanced matching algorithms that pair contributors to customers for optimal turnaround and accuracy
+- Create optimized and efficient UI/UX tooling, in combination with ML algorithms, for 100k+ contributors completing billions of complex tasks
+- Develop new AI infrastructure products to visualize, query, and explore Scale data
+- Build a customer service RAG application that handles thousands of questions a day
+- Integrate a cutting-edge ML model that predicts churn into a customer's retention system
+Qualification:
+Full-Stack Web Development, API Integration, Large-Scale Data Processing, Python, TypeScript, React, MongoDB, Large-Scale Product Engineering, Large Language Models (LLMs), LLM Evaluation, Agentic Systems
+Required:
+- A graduation date in Fall 2026 or Spring 2027 with a Bachelor's degree (or equivalent) in a relevant field (Computer Science, EECS, Computer Engineering, Statistics)
+- Product engineering experience such as building web apps full-stack, integrating with relevant APIs and services, talking to customers, figuring out 'what' to build and then iterating
+- Previous Product/Software Engineering internship experience
+- Track record of shipping high-quality products and features at scale
+- Experience building systems that process large volumes of data
+- Experience with Python, Typescript, React, and/or MongoDB
+Preferred:
+- Hands-on experience with LLMs, evaluations, or agentic systems — whether from internships, research, or personal projects
+- Open source contributions or a portfolio of shipped side projects
+Benefits:
+- Base salary, equity, and benefits
+- Comprehensive health, dental and vision coverage
+- Retirement benefits
+- A learning and development stipend
+- Generous PTO
+- This role may be eligible for a commuter stipend</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>New Grad</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>2026-09-09 01:54:26</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>JobRight</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>Gmail from no-reply@us.greenhouse-mail.io subject 'Thank you for applying to Scale AI' dated 2026-09-09 states 'Your application has been received' for Scale AI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>url:fd9e6f8d3d7738566389</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Software Engineer - New Grad (2027)</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Replit</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Foster City, CA</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/replit/b5e81eae-06f9-4798-8988-2d06ca936dbc/application?jr_id=6aa1ad3a3272060a8e3f17a8</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>$140K – $180K</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Software Engineer - New Grad (2027)
+Location: Foster City, CA
+Employment Type: Full time
+Location Type: Hybrid
+Department: Engineering - Early Career
+Compensation: Compensation is determined based on career level, with the base salary for this role ranging from $140K – $180K • Offers Equity • Offers Bonus • Performance Based Bonus</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>2026-09-09 23:31:22</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Ashby</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>Confirmation email from Replit Hiring Team (via Ashby) states received application for Software Engineer (New Grad 2027) role.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>

<commit_message>
Improved the prompts to customize the resume and answer experience questions
</commit_message>
<xml_diff>
--- a/data/applied_jobs.xlsx
+++ b/data/applied_jobs.xlsx
@@ -446,12 +446,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V54"/>
+  <dimension ref="A1:V72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="33.85714285714285" customWidth="1" min="1" max="1"/>
     <col width="42.14285714285715" customWidth="1" min="2" max="2"/>
-    <col width="13.57142857142857" customWidth="1" min="3" max="8"/>
+    <col width="28.28571428571428" customWidth="1" min="3" max="3"/>
+    <col width="13.57142857142857" customWidth="1" min="4" max="8"/>
     <col width="39" customWidth="1" min="9" max="9"/>
     <col width="13.57142857142857" customWidth="1" min="10" max="24"/>
   </cols>
@@ -2528,134 +2529,40 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>url:74234e98afe7498fb5da</t>
+          <t>url:459f24387c0c3190776f</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>AI Associate</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Adobe</t>
+          <t>Alumni Ventures</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>Manchester, New Hampshire, USA</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>5 hours ago</t>
+          <t>null</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>https://job-boards.greenhouse.io/embed/job_app?for=alumniventures&amp;token=4299342009&amp;jr_id=6a8c5b5fcde3717f9e9bc921</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>$126K/yr - $234K/yr</t>
+          <t>null</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
-        <is>
-          <t>Adobe is a company that provides digital experience, creative, and cloud solutions powered by AI. The Machine Learning Engineer will develop machine learning models and algorithms for search, discovery, recommendations, content understanding, and generative AI, while building scalable machine learning services for Adobe Cloud assets.
-Responsibilities
-Build novel machine learning models using deep learning, reinforcement learning, content understanding, language understanding, and more by developing pioneering machine learning algorithms for Search&amp;Discovery team
-Apply machine learning/reinforcement learning to improve content understanding, computer vision, deep learning, language understanding and content ranking &amp; recommendations
-Build machine learning offerings to enable lifecycle of billions of images, documents and other assets in Adobe Cloud
-Build machine learning services to host AI/ML models using technologies such as REST web services, micro-services, machine learning frameworks, Pytorch, Tensorflow, and LLMs
-Qualification
-Required
-* Good understanding of statistical modeling, machine learning, deep learning, or data analytics concepts
-* Proficient in one or more programming languages such as Python, Java and C
-* Familiar with one or more machine learning or statistical modeling tools such as PyTorch, SGLang, Verl and scikit learn
-* Strong analytical and quantitative problem-solving ability
-* Excellent communication, relationship skills and a great teammate
-Preferred
-* MS/PhD (preferred) in Computer Science, Machine Learning or equivalent field
-Benefits
-Non-sales roles starting salaries are expressed as base salary and short-term incentives are in the form of the Annual Incentive Plan (AIP).
-Certain roles may be eligible for long-term incentives in the form of a new hire equity award.</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>Entry Level</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>Full-time</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>2026-09-11 00:42:44</t>
-        </is>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>Jobright</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>Gmail had no Levelpath confirmation email. Application page shows Success: Your application was successfully submitted for AI Solutions Specialist at Levelpath.</t>
-        </is>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>Employer explicitly states OPT/STEM OPT cannot be supported: 'GM does not provide immigration-related sponsorship for this role... (e.g., H1-B, OPT, STEM OPT, CPT, TN, J-1, etc.)'</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>url:459f24387c0c3190776f</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>AI Associate</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Alumni Ventures</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Manchester, New Hampshire, USA</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/embed/job_app?for=alumniventures&amp;token=4299342009&amp;jr_id=6a8c5b5fcde3717f9e9bc921</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
         <is>
           <t>AI Associate
 Manchester, New Hampshire, USA
@@ -2715,6 +2622,78 @@
 This position requires working onsite at our Manchester, NH office Monday through Friday.</t>
         </is>
       </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>2026-09-07 20:03:27</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Greenhouse</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Greenhouse confirmation email from no-reply@us.greenhouse-mail.io confirms application to Alumni Ventures for AI Associate and states team will review application.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>url:c20e4e44e3e864da48d7</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Baseten</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/baseten/ae64d1d4-7b0a-4be4-8d77-7f5ce63849a7/application?jr_id=6a0fd9af12f8b43cf3981fe0</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
       <c r="J27" t="inlineStr">
         <is>
           <t>null</t>
@@ -2732,39 +2711,39 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>2026-09-07 20:03:27</t>
+          <t>2026-09-07 20:32:25</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>Ashby</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>Greenhouse confirmation email from no-reply@us.greenhouse-mail.io confirms application to Alumni Ventures for AI Associate and states team will review application.</t>
+          <t>Found matching confirmation email from Baseten Hiring Team via Ashby ATS confirming application for Software Engineer - Infrastructure role was received and will be reviewed.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>url:c20e4e44e3e864da48d7</t>
+          <t>url:6eb94343ec86d204c1c8</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>ML Engineer</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Baseten</t>
+          <t>Catalyst Labs</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Sunnyvale, California, United States</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2774,87 +2753,15 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/baseten/ae64d1d4-7b0a-4be4-8d77-7f5ce63849a7/application?jr_id=6a0fd9af12f8b43cf3981fe0</t>
+          <t>https://www.careers-page.com/catalyst-labs/job/8XX35V7R?jr_id=6a58ca0c3ac7627fe9ffb490</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>above market base + bonus + equity</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>2026-09-07 20:32:25</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>Ashby</t>
-        </is>
-      </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>Found matching confirmation email from Baseten Hiring Team via Ashby ATS confirming application for Software Engineer - Infrastructure role was received and will be reviewed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>url:6eb94343ec86d204c1c8</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>ML Engineer</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Catalyst Labs</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Sunnyvale, California, United States</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>https://www.careers-page.com/catalyst-labs/job/8XX35V7R?jr_id=6a58ca0c3ac7627fe9ffb490</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>above market base + bonus + equity</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
         <is>
           <t>ML Engineer
 Sunnyvale, California, United States
@@ -2894,6 +2801,78 @@
 Solid grasp of ML systems architecture, feature engineering, evaluation strategies, and deployment best practices.</t>
         </is>
       </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>2026-09-07 20:36:21</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>careers-page.com</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Page shows 'Thank you for your application! Your application was successfully submitted.' for ML Engineer at Catalyst Labs; no qualifying confirmation email found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>lever:401c169a-5b21-4dda-a65b-ac78c2f4e605:apply</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>AI/ML Data Contributor</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>TSMG</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Oklahoma City, OK, Remote</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/tsmg/401c169a-5b21-4dda-a65b-ac78c2f4e605/apply?jr_id=6a5d49d8856af468ab010921</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
       <c r="J29" t="inlineStr">
         <is>
           <t>null</t>
@@ -2901,7 +2880,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Full Time</t>
+          <t>Contract Full Time</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -2911,39 +2890,39 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>2026-09-07 20:36:21</t>
+          <t>2026-09-07 20:47:21</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>careers-page.com</t>
+          <t>Lever</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>Page shows 'Thank you for your application! Your application was successfully submitted.' for ML Engineer at Catalyst Labs; no qualifying confirmation email found.</t>
+          <t>Gmail confirmation from TSMG via Lever states application received for AI/ML Data Contributor.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>lever:401c169a-5b21-4dda-a65b-ac78c2f4e605:apply</t>
+          <t>url:3dacb6e26da529cb73a4</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AI/ML Data Contributor</t>
+          <t>Data Engineer</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>TSMG</t>
+          <t>Sedgwick</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, Remote</t>
+          <t>Telecommuter-FL</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2953,7 +2932,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/tsmg/401c169a-5b21-4dda-a65b-ac78c2f4e605/apply?jr_id=6a5d49d8856af468ab010921</t>
+          <t>https://sedgwick.wd1.myworkdayjobs.com/sedgwick/job/Telecommuter-FL/Data-Engineer_R71134-1?jr_id=6a9622b84c22023a0793848b</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2973,7 +2952,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Contract Full Time</t>
+          <t>null</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -2983,39 +2962,39 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>2026-09-07 20:47:21</t>
+          <t>2026-09-07 20:57:17</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Lever</t>
+          <t>Workday</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>Gmail confirmation from TSMG via Lever states application received for AI/ML Data Contributor.</t>
+          <t>Gmail had no qualifying confirmation email. Application site shows 'Application Submitted' dialog stating 'You have successfully completed your application!' for Sedgwick.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>url:3dacb6e26da529cb73a4</t>
+          <t>url:b95bddf301326465a7b9</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Data Engineer</t>
+          <t>Forward Deployed Engineer (AI Solutions) - NA East Market</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Sedgwick</t>
+          <t>Aircall</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Telecommuter-FL</t>
+          <t>New York Office</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3025,87 +3004,15 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://sedgwick.wd1.myworkdayjobs.com/sedgwick/job/Telecommuter-FL/Data-Engineer_R71134-1?jr_id=6a9622b84c22023a0793848b</t>
+          <t>https://job-boards.greenhouse.io/embed/job_app?for=aircallioinc&amp;token=4308436009&amp;jr_id=6a7a562967a1ad0bc53d302e</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>$120,000 - $190,000 a year</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>2026-09-07 20:57:17</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>Workday</t>
-        </is>
-      </c>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>Gmail had no qualifying confirmation email. Application site shows 'Application Submitted' dialog stating 'You have successfully completed your application!' for Sedgwick.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>url:b95bddf301326465a7b9</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Forward Deployed Engineer (AI Solutions) - NA East Market</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Aircall</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>New York Office</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/embed/job_app?for=aircallioinc&amp;token=4308436009&amp;jr_id=6a7a562967a1ad0bc53d302e</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>$120,000 - $190,000 a year</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
         <is>
           <t>Forward Deployed Engineer (AI Solutions) - NA East Market
 New York Office
@@ -3176,74 +3083,74 @@
 We may use artificial intelligence (AI) tools to support parts of the hiring process, such as reviewing applications, analyzing resumes, or assessing responses. These tools assist our recruitment team but do not replace human judgment. Final hiring decisions are ultimately made by humans. If you would like more information about how your data is processed, please contact us.</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>2026-09-07 22:18:10</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t>Greenhouse</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
+      <c r="P31" t="inlineStr">
         <is>
           <t>Greenhouse confirmation page states 'Thank you for applying. Your application has been received.' for Aircall. No qualifying Gmail confirmation found.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>url:6997c4fe682d26534797</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>Forward Deployed Engineer (AI Solutions) - NA East Market</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>Aircall</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>New York Office</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/embed/job_app?for=aircallioinc&amp;token=4308436009&amp;jr_id=6a7a562967a1ad0bc53d302e&amp;utm_source=Simplify&amp;gh_src=Simplify</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>$120,000 - $190,000 a year</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>Forward Deployed Engineer (AI Solutions) - NA East Market
 New York Office
@@ -3302,69 +3209,69 @@
 DE&amp;I Statement: At Aircall, we believe diversity, equity and inclusion – irrespective of origins, identity, background and orientations – are core to our journey. We pride ourselves on promoting active inclusion within our business to foster a strong sense of belonging for all. We're working to create a place filled with diverse people who can enrich and learn from one another. We're committed to ensuring that everyone not only has a seat at the table but is valued and respected at it by providing equal opportunities to develop and thrive.</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>2026-09-07 22:13:27</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
+      <c r="N32" t="inlineStr">
         <is>
           <t>Greenhouse</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>url:11429f1f5d340566c153</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>AI Engineer</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>Stripe</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>Toronto, Atlanta, Chicago</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
         <is>
           <t>https://stripe.com/careers/listing/ai-engineer/8044460?gh_src=73vnei</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>$126,600 - $189,800</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>AI Engineer
 Who We Are
@@ -3422,6 +3329,78 @@
 At Stripe, we're looking for people with passion, grit, and integrity. You're encouraged to apply even if your experience doesn't precisely match the job description. Your skills and passion will stand out—and set you apart—especially if your career has taken some extraordinary twists and turns. At Stripe, we welcome diverse perspectives and people who think rigorously and aren't afraid to challenge assumptions. Join us.</t>
         </is>
       </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>2026-09-07 22:36:16</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Stripe confirmation email from no-reply@stripe.com confirms submission for AI Engineer role: 'Thanks so much for submitting your application'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>url:c2077b5e6cf0e66571c9</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Data Scientist</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>https://evlo.ai/jobs/apply/bf-g0051-s06?utm_content=bf-g0051-s06&amp;utm_term=ai-machine-learning&amp;utm_campaign=bluefunnel&amp;utm_source=linkedin&amp;src=LinkedIn-bluefunnel</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
       <c r="J34" t="inlineStr">
         <is>
           <t>null</t>
@@ -3429,17 +3408,17 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Full time</t>
+          <t>null</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Applied</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>2026-09-07 22:36:16</t>
+          <t>2026-09-07 22:12:10</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -3449,29 +3428,34 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>Stripe confirmation email from no-reply@stripe.com confirms submission for AI Engineer role: 'Thanks so much for submitting your application'.</t>
+          <t>No qualifying Gmail confirmation for evlo/Data Scientist found. evlo.ai shows Data Scientist role with Apply button but no submission confirmation, receipt, error, or CAPTCHA.</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>No qualifying Gmail confirmation for evlo/Data Scientist found. evlo.ai shows Data Scientist role with Apply button but no submission confirmation, receipt, error, or CAPTCHA.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>url:c2077b5e6cf0e66571c9</t>
+          <t>url:a0f9cbfd23822145dda1</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Software Engineer</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Applied Intuition</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Sunnyvale</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -3481,12 +3465,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://evlo.ai/jobs/apply/bf-g0051-s06?utm_content=bf-g0051-s06&amp;utm_term=ai-machine-learning&amp;utm_campaign=bluefunnel&amp;utm_source=linkedin&amp;src=LinkedIn-bluefunnel</t>
+          <t>https://jobs.ashbyhq.com/applied/43286c63-937d-4384-a5ff-12cb31baa225/application?jr_id=6a7e4c120cd4a0703257f2ca</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>$182.6K – $243.9K • Offers Equity</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3501,54 +3485,44 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Full time</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Not Applied</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>2026-09-07 22:12:10</t>
+          <t>2026-09-09 23:53:11</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t>No qualifying Gmail confirmation for evlo/Data Scientist found. evlo.ai shows Data Scientist role with Apply button but no submission confirmation, receipt, error, or CAPTCHA.</t>
-        </is>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>No qualifying Gmail confirmation for evlo/Data Scientist found. evlo.ai shows Data Scientist role with Apply button but no submission confirmation, receipt, error, or CAPTCHA.</t>
+          <t>Ashby</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>url:a0f9cbfd23822145dda1</t>
+          <t>url:5774cdf89f5e667098e7</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Software Engineer</t>
+          <t>Software Engineer, Inference AI/ML</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Applied Intuition</t>
+          <t>CoreWeave</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Sunnyvale</t>
+          <t>Sunnyvale, CA / Bellevue, WA</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -3558,82 +3532,15 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/applied/43286c63-937d-4384-a5ff-12cb31baa225/application?jr_id=6a7e4c120cd4a0703257f2ca</t>
+          <t>https://job-boards.greenhouse.io/embed/job_app?for=coreweave&amp;token=4609928006&amp;jr_id=6a9fee1036c44a0fd09b8ed1</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>$182.6K – $243.9K • Offers Equity</t>
+          <t>$92,000 to $135,000</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>2026-09-09 23:53:11</t>
-        </is>
-      </c>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>Ashby</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>url:5774cdf89f5e667098e7</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Software Engineer, Inference AI/ML</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>CoreWeave</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Sunnyvale, CA / Bellevue, WA</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/embed/job_app?for=coreweave&amp;token=4609928006&amp;jr_id=6a9fee1036c44a0fd09b8ed1</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>$92,000 to $135,000</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
         <is>
           <t>CoreWeave is The Essential Cloud for AI™. Built for pioneers by pioneers, CoreWeave delivers a platform of technology, tools, and teams that enables innovators to build and scale AI with confidence. Trusted by leading AI labs, startups, and global enterprises, CoreWeave combines superior infrastructure performance with deep technical expertise to accelerate breakthroughs and turn compute into capability. Founded in 2017, CoreWeave became a publicly traded company (Nasdaq: CRWV) in March 2025. Learn more at www.coreweave.com.
 What You’ll Do:
@@ -3667,74 +3574,74 @@
 CoreWeave is an equal opportunity employer, committed to fostering an inclusive and supportive workplace. All qualified applicants and candidates will receive consideration for employment without regard to race, color, religion, sex, disability, age, sexual orientation, gender identity, national origin, veteran status, or genetic information.</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
+      <c r="M36" t="inlineStr">
         <is>
           <t>2026-09-08 10:51:48</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr">
+      <c r="N36" t="inlineStr">
         <is>
           <t>Greenhouse</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr">
+      <c r="P36" t="inlineStr">
         <is>
           <t>Greenhouse confirmation page states 'Thank you for your applying to CoreWeave. Your application is under review.' No qualifying Gmail confirmation email found.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t>url:a4797e18694697c98a0a</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>Machine Learning Engineer, Tapestry</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>Tapestry</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>Mountain View, CA (HQ)</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
         <is>
           <t>https://boards.greenhouse.io/embed/job_app?token=8722582002&amp;jr_id=6a8378f0379c304e892f7967</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>$166,000 - $244,000 + bonus + equity + benefits</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>About Tapestry
 Tapestry is a group within Google working to build the AI-powered electric grid. We are tackling one of the world’s most important infrastructure challenges: helping the energy system become more visible, understandable, reliable, affordable, abundant, and clean.
@@ -3776,6 +3683,83 @@
 Please note that the compensation details listed in US role postings reflect the base salary only, and do not include bonus, equity, or benefits.</t>
         </is>
       </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>2026-09-09 23:50:10</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Greenhouse</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Gmail confirmation from careers-no-reply@x.team confirms receipt of application for Machine Learning Engineer, Tapestry position at X.</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Application was not submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>url:9d4f74b3010c055ac558</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>CATT Technical Delivery AI Software Engineer - Fall 2027</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>RSM</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Atlanta Metro Area</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://rsm.wd1.myworkdayjobs.com/en-US/RSMCareers/job/Atlanta-Metro-Area/CATT-Technical-Delivery-AI-Software-Engineer---Fall-2027_JR121013/apply/applyManually</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
       <c r="J38" t="inlineStr">
         <is>
           <t>null</t>
@@ -3783,7 +3767,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Full-time</t>
+          <t>null</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -3793,44 +3777,39 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>2026-09-09 23:50:10</t>
+          <t>2026-09-08 11:21:15</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>Workday</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>Gmail confirmation from careers-no-reply@x.team confirms receipt of application for Machine Learning Engineer, Tapestry position at X.</t>
-        </is>
-      </c>
-      <c r="Q38" t="inlineStr">
-        <is>
-          <t>Application was not submitted.</t>
+          <t>Confirmation email from rsm@myworkday.com with subject 'Thank you for applying to RSM!' names the CATT Technical Delivery AI Software Engineer - Fall 2027 role and states application status can be checked in applicant profile.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>url:9d4f74b3010c055ac558</t>
+          <t>url:34e4217a5c7c7dff852d</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>CATT Technical Delivery AI Software Engineer - Fall 2027</t>
+          <t>null</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>RSM</t>
+          <t>Roblox</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Atlanta Metro Area</t>
+          <t>null</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3840,7 +3819,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://rsm.wd1.myworkdayjobs.com/en-US/RSMCareers/job/Atlanta-Metro-Area/CATT-Technical-Delivery-AI-Software-Engineer---Fall-2027_JR121013/apply/applyManually</t>
+          <t>https://job-boards.greenhouse.io/embed/job_app?for=roblox&amp;jr_id=6a836d9fb5a0ac0e84a25b2a&amp;token=8123004</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3870,129 +3849,57 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>2026-09-08 11:21:15</t>
+          <t>2026-09-08 11:44:02</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>Workday</t>
+          <t>Greenhouse</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>Confirmation email from rsm@myworkday.com with subject 'Thank you for applying to RSM!' names the CATT Technical Delivery AI Software Engineer - Fall 2027 role and states application status can be checked in applicant profile.</t>
+          <t>Greenhouse page shows 'Thank you for applying to Roblox!' and 'Your application has been received.' No qualifying Gmail confirmation found.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>url:34e4217a5c7c7dff852d</t>
+          <t>url:e85ba8d9364022692844</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Associate Data Scientist</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Roblox</t>
+          <t>Capgemini</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Houston, TX, US</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Sep 1, 2026</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/embed/job_app?for=roblox&amp;jr_id=6a836d9fb5a0ac0e84a25b2a&amp;token=8123004</t>
+          <t>https://careers.capgemini.com/job/Houston%2C-TX-Associate-Data-Scientist-TX-77001/1432707133/?from=email&amp;refid=31456055801&amp;utm_source=J2WEmail&amp;source=2&amp;eid=219901-202633080233-34979178101&amp;locale=en_US</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>$70,000- $105,000</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>2026-09-08 11:44:02</t>
-        </is>
-      </c>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>Greenhouse</t>
-        </is>
-      </c>
-      <c r="P40" t="inlineStr">
-        <is>
-          <t>Greenhouse page shows 'Thank you for applying to Roblox!' and 'Your application has been received.' No qualifying Gmail confirmation found.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>url:e85ba8d9364022692844</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Associate Data Scientist</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Capgemini</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Houston, TX, US</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Sep 1, 2026</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>https://careers.capgemini.com/job/Houston%2C-TX-Associate-Data-Scientist-TX-77001/1432707133/?from=email&amp;refid=31456055801&amp;utm_source=J2WEmail&amp;source=2&amp;eid=219901-202633080233-34979178101&amp;locale=en_US</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>$70,000- $105,000</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
         <is>
           <t>Associate Data Scientist
 Choosing Capgemini means choosing a company where you will be empowered to shape your career in the way you'd like, where you'll be supported and inspired by a collaborative community of colleagues around the world, and where you'll be able to reimagine what's possible. Join us and help the world's leading organizations unlock the value of technology and build a more sustainable, more inclusive world.
@@ -4035,74 +3942,74 @@
 Nearest Major Market: Houston</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="J40" t="inlineStr">
         <is>
           <t>Experienced Professionals</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="K40" t="inlineStr">
         <is>
           <t>Permanent</t>
         </is>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="L40" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
+      <c r="M40" t="inlineStr">
         <is>
           <t>2026-09-08 12:55:47</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr">
+      <c r="N40" t="inlineStr">
         <is>
           <t>Capgemini</t>
         </is>
       </c>
-      <c r="P41" t="inlineStr">
+      <c r="P40" t="inlineStr">
         <is>
           <t>Confirmation email from HRsystem@capgemini.com with subject 'Capgemini Group – New Job Application Received' confirms receipt of Associate Data Scientist application.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t>url:d4ad477a97298d95468e</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>Associate-AI-ML Engineer / GenAI Engineer - Data Scientist</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>Capgemini</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>Houston, TX, US - Onsite</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>Sep 3, 2026</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G41" t="inlineStr">
         <is>
           <t>https://careers.capgemini.com/job/Houston%2C-TX-Associate-AI-ML-Engineer-GenAI-Engineer-Data-Scientist-TX-77001/1433639533/?from=email&amp;refid=31456055801&amp;utm_source=J2WEmail&amp;source=2&amp;eid=219901-202633080233-34979178101&amp;locale=en_US</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H41" t="inlineStr">
         <is>
           <t>$46,000 to $111,000</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>Associate-AI-ML Engineer / GenAI Engineer - Data Scientist
 Choosing Capgemini means choosing a company where you will be empowered to shape your career in the way you'd like, where you'll be supported and inspired by a collaborative community of colleagues around the world, and where you'll be able to reimagine what's possible. Join us and help the world's leading organizations unlock the value of technology and build a more sustainable, more inclusive world.
@@ -4147,74 +4054,74 @@
 Nearest Major Market: Houston</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="J41" t="inlineStr">
         <is>
           <t>Experienced Professionals</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="K41" t="inlineStr">
         <is>
           <t>Permanent</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="L41" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="M41" t="inlineStr">
         <is>
           <t>2026-09-08 13:14:22</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr">
+      <c r="N41" t="inlineStr">
         <is>
           <t>Capgemini</t>
         </is>
       </c>
-      <c r="P42" t="inlineStr">
+      <c r="P41" t="inlineStr">
         <is>
           <t>Gmail from HRsystem@capgemini.com 'Capgemini Group – New Job Application Received' confirms application for Associate-AI-ML Engineer / GenAI Engineer - Data Scientist received and under review.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
+    <row r="42">
+      <c r="A42" t="inlineStr">
         <is>
           <t>url:5fd52c75ef50687b6ac7</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>Junior Analyst - AI Solutions, R&amp;D &amp; Coding</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>StepStone Group</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>La Jolla</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/embed/job_app?for=stepstone&amp;token=8171272&amp;jr_id=6aa0360fea127c3794695824</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H42" t="inlineStr">
         <is>
           <t>$29.00/Hour</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>We are global private markets specialists delivering tailored investment solutions, advisory services, and impactful, data driven insights to the world's investors. Leveraging the power of our platform and our peerless intelligence across sectors, strategies, and geographies, we help identify the advantages and the answers our clients need to succeed.
 Position Overview
@@ -4247,74 +4154,74 @@
 Candidates must be at least 18 years old to apply.</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
+      <c r="M42" t="inlineStr">
         <is>
           <t>2026-09-08 13:22:35</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr">
+      <c r="N42" t="inlineStr">
         <is>
           <t>Greenhouse</t>
         </is>
       </c>
-      <c r="P43" t="inlineStr">
+      <c r="P42" t="inlineStr">
         <is>
           <t>Greenhouse confirmation page states 'Thank you for applying. Your application has been received.' No qualifying confirmation email found.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
+    <row r="43">
+      <c r="A43" t="inlineStr">
         <is>
           <t>url:0d1b155982fabe32a612</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>AI Engineer – Center of Excellence</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>Aderant</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>Atlanta, GA</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>2 hours ago</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t>https://jobright.ai/jobs/info/6a985e88c8ed473c5c763af1</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
         <is>
           <t>Aderant is a software company providing business management solutions for law firms and other professional services organizations. The AI Engineer will design, develop, and deploy scalable AI-powered solutions, including machine learning and generative AI systems, and integrate them into business applications. The role also involves collaborating with product and engineering teams, monitoring model performance, and supporting enterprise-wide AI adoption.
 Responsibilities:
@@ -4337,74 +4244,74 @@
 Benefits: Hybrid work arrangement</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="J43" t="inlineStr">
         <is>
           <t>Entry Level</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="K43" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr">
+      <c r="L43" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr">
+      <c r="M43" t="inlineStr">
         <is>
           <t>2026-09-08 13:37:02</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr">
+      <c r="N43" t="inlineStr">
         <is>
           <t>JobRight</t>
         </is>
       </c>
-      <c r="P44" t="inlineStr">
+      <c r="P43" t="inlineStr">
         <is>
           <t>Gmail from aderant@myworkday.com subject 'Application Received for AI Engineer – Center of Excellence' confirms: Thank you for your application for AI Engineer – Center of Excellence at Aderant.</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t>url:113d46a46c7e86a603c5</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>AI Engineer</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>Infosys</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>Hartford, CT</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>4 hours ago</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G44" t="inlineStr">
         <is>
           <t>https://jobright.ai/jobs/info/6a84a2727b33d722762572e7</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
         <is>
           <t>Infosys is a global leader in next-generation digital services and consulting. The AI Engineer role focuses on data preparation, statistical and machine learning model development, generative AI, model validation, and deployment of analytics solutions. The role also involves collaborating with business and technology teams, documenting model activities, and ensuring data and operational quality.
 Responsibilities:
@@ -4444,74 +4351,74 @@
 - Paid holidays plus Paid Time Off</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="J44" t="inlineStr">
         <is>
           <t>Entry Level</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="K44" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr">
+      <c r="L44" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr">
+      <c r="M44" t="inlineStr">
         <is>
           <t>2026-09-08 22:12:32</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr">
+      <c r="N44" t="inlineStr">
         <is>
           <t>JobRight</t>
         </is>
       </c>
-      <c r="P45" t="inlineStr">
+      <c r="P44" t="inlineStr">
         <is>
           <t>Confirmation page shows 'Thank you for your submission!' for Infosys AI Engineer with instructions to check candidate zone. No qualifying Gmail confirmation email found.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
+    <row r="45">
+      <c r="A45" t="inlineStr">
         <is>
           <t>url:2245f9f895023899a9a0</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>Associate Data Engineer</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>Infoblox</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>Tacoma, WA</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>43 minutes ago</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="G45" t="inlineStr">
         <is>
           <t>https://jobright.ai/jobs/info/6aa09854dbc0e60e37e0ea80</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
         <is>
           <t>Infoblox is a provider of cloud-first networking and security solutions. The company is seeking an Associate Data Engineer to curate and deliver high-quality data for data-driven insights, threat analytics, and business and product decisions. The role focuses on building scalable data pipelines and platforms, supporting data science and AI/ML applications, and collaborating with engineering teams to operationalize AI solutions.
 Responsibilities:
@@ -4556,74 +4463,74 @@
 - Corporate bonus</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="J45" t="inlineStr">
         <is>
           <t>Entry Level</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
+      <c r="L45" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr">
+      <c r="M45" t="inlineStr">
         <is>
           <t>2026-09-08 22:30:58</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr">
+      <c r="N45" t="inlineStr">
         <is>
           <t>Jobright</t>
         </is>
       </c>
-      <c r="P46" t="inlineStr">
+      <c r="P45" t="inlineStr">
         <is>
           <t>Gmail from Infoblox Careers confirms application for Associate Data Engineer - 7837: 'Thank you for taking the time to apply... We will review your application.'</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t>url:3025b0ba356efc6a731c</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>Software Engineer - New Grad</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>Scale AI</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>San Francisco, CA</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t>2 days ago</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="G46" t="inlineStr">
         <is>
           <t>https://jobright.ai/jobs/info/6a9af73bd5ff1f3f1c39caae</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="H46" t="inlineStr">
         <is>
           <t>$124K/yr - $162K/yr</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>Scale AI develops reliable AI systems, data, and full-stack technologies that support leading models and enterprise and government applications. The New Grad Software Engineer will own customer-facing product engineering work, shipping and iterating on AI products, data systems, applications, and infrastructure at scale.
 Responsibilities:
@@ -4659,74 +4566,74 @@
 - This role may be eligible for a commuter stipend</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="J46" t="inlineStr">
         <is>
           <t>New Grad</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="K46" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr">
+      <c r="L46" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr">
+      <c r="M46" t="inlineStr">
         <is>
           <t>2026-09-09 01:54:26</t>
         </is>
       </c>
-      <c r="N47" t="inlineStr">
+      <c r="N46" t="inlineStr">
         <is>
           <t>JobRight</t>
         </is>
       </c>
-      <c r="P47" t="inlineStr">
+      <c r="P46" t="inlineStr">
         <is>
           <t>Gmail from no-reply@us.greenhouse-mail.io subject 'Thank you for applying to Scale AI' dated 2026-09-09 states 'Your application has been received' for Scale AI.</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t>url:fd9e6f8d3d7738566389</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>Software Engineer - New Grad (2027)</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>Replit</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>Foster City, CA</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/replit/b5e81eae-06f9-4798-8988-2d06ca936dbc/application?jr_id=6aa1ad3a3272060a8e3f17a8</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
+      <c r="H47" t="inlineStr">
         <is>
           <t>$140K – $180K</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>Software Engineer - New Grad (2027)
 Location: Foster City, CA
@@ -4736,74 +4643,74 @@
 Compensation: Compensation is determined based on career level, with the base salary for this role ranging from $140K – $180K • Offers Equity • Offers Bonus • Performance Based Bonus</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
         <is>
           <t>Full time</t>
         </is>
       </c>
-      <c r="L48" t="inlineStr">
+      <c r="L47" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr">
+      <c r="M47" t="inlineStr">
         <is>
           <t>2026-09-09 23:31:22</t>
         </is>
       </c>
-      <c r="N48" t="inlineStr">
+      <c r="N47" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
       </c>
-      <c r="P48" t="inlineStr">
+      <c r="P47" t="inlineStr">
         <is>
           <t>Confirmation email from Replit Hiring Team (via Ashby) states received application for Software Engineer (New Grad 2027) role.</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>url:b25d7ab7a4f2423506d4</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>AI Software Engineer</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>Relativity Space</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>Long Beach, CA</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F48" t="inlineStr">
         <is>
           <t>15 hours ago</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
+      <c r="G48" t="inlineStr">
         <is>
           <t>https://jobright.ai/jobs/info/6a84b3a42f4f0014cae2241b</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="H48" t="inlineStr">
         <is>
           <t>$115K/yr - $173K/yr</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="I48" t="inlineStr">
         <is>
           <t>Relativity Space is building rockets and an automated rocket factory to support current and future space missions. The AI Software Engineer will build and iterate on AI-powered applications and agents for engineers and operators, contributing across the full software development life cycle. The role also involves collaborating with users and stakeholders, applying agile practices, and delivering reliable production software.
 Responsibilities:
@@ -4833,74 +4740,74 @@
 Experience: 1+ years exp</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="J48" t="inlineStr">
         <is>
           <t>Entry Level</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
       </c>
-      <c r="L49" t="inlineStr">
+      <c r="L48" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr">
+      <c r="M48" t="inlineStr">
         <is>
           <t>2026-09-10 01:32:59</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr">
+      <c r="N48" t="inlineStr">
         <is>
           <t>JobRight</t>
         </is>
       </c>
-      <c r="P49" t="inlineStr">
+      <c r="P48" t="inlineStr">
         <is>
           <t>Greenhouse confirmation email from no-reply@us.greenhouse-mail.io dated 2026-09-10 for Relativity Space states application received for AI Software Engineer.</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>url:8b0799946b15885d2e6f</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>AI Software Engineer</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>Relativity Space</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>Long Beach, California, United States</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/embed/job_app?for=relativity&amp;jr_id=6a84b3a42f4f0014cae2241b&amp;token=8726261002&amp;utm_source=Simplify&amp;gh_src=Simplify</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="H49" t="inlineStr">
         <is>
           <t>$115,000 - $173,000 USD</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>AI Software Engineer
 Long Beach, California, United States
@@ -4932,74 +4839,74 @@
 We are an equal opportunity employer and value diversity at our company. We do not discriminate on the basis of race, religion, color, national origin, gender, sexual orientation, age, marital status, veteran status, or disability status.</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
       </c>
-      <c r="L50" t="inlineStr">
+      <c r="L49" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr">
+      <c r="M49" t="inlineStr">
         <is>
           <t>2026-09-10 01:24:28</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr">
+      <c r="N49" t="inlineStr">
         <is>
           <t>Greenhouse</t>
         </is>
       </c>
-      <c r="P50" t="inlineStr">
+      <c r="P49" t="inlineStr">
         <is>
           <t>Greenhouse confirmation page for Relativity Space shows 'Thank you for applying. Your application has been received.' No qualifying confirmation email found.</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>url:b6b45a06e5cecbae7a3f</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>Machine Learning Software Engineer 1</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>Crowe</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>Chicago, IL</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>13 hours ago</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
+      <c r="G50" t="inlineStr">
         <is>
           <t>https://jobright.ai/jobs/info/6a7f6404ad9ff00c26baded5</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
+      <c r="H50" t="inlineStr">
         <is>
           <t>$62K/yr - $100K/yr</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr">
+      <c r="I50" t="inlineStr">
         <is>
           <t>Crowe provides audit, tax, advisory, consulting, and other professional services. The Machine Learning Software Engineer 1 develops reusable libraries and services for machine learning products, collaborates with data scientists to move models from prototype to production, and supports software development throughout the project lifecycle.
 Responsibilities
@@ -5038,141 +4945,141 @@
 Equitable access to opportunities for career growth and leadership</t>
         </is>
       </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Entry Level</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>2026-09-10 01:43:38</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>JobRight</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>url:a39131e8099736db65d0</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Machine Learning Software Engineer 1</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Crowe</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Chicago, IL, USA</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://crowe.wd12.myworkdayjobs.com/en-US/external_careers/job/Chicago-IL-USA/Machine-Learning-Software-Engineer-1_R-71006/apply/applyManually</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Entry Level</t>
+          <t>null</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>Full-time</t>
+          <t>null</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Not Applied</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>2026-09-10 01:43:38</t>
+          <t>2026-09-10 01:54:30</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>JobRight</t>
+          <t>Workday</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Found Workday @ Crowe email 'Thank You For Applying!' confirming completed application for Machine Learning Software Engineer 1 role at Crowe.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>url:a39131e8099736db65d0</t>
+          <t>url:efb7647fedee09052b11</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Machine Learning Software Engineer 1</t>
+          <t>LLM – AI Quality Analyst</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Crowe</t>
+          <t>RLink Solutions</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Chicago, IL, USA</t>
+          <t>United States, Remote</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>7 hours ago</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://crowe.wd12.myworkdayjobs.com/en-US/external_careers/job/Chicago-IL-USA/Machine-Learning-Software-Engineer-1_R-71006/apply/applyManually</t>
+          <t>https://jobright.ai/jobs/info/6aa1f5772f936e4a53daee7c</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>$25/hr - $30/hr</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>2026-09-10 01:54:30</t>
-        </is>
-      </c>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>Workday</t>
-        </is>
-      </c>
-      <c r="P52" t="inlineStr">
-        <is>
-          <t>Found Workday @ Crowe email 'Thank You For Applying!' confirming completed application for Machine Learning Software Engineer 1 role at Crowe.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>url:efb7647fedee09052b11</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>LLM – AI Quality Analyst</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>RLink Solutions</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>United States, Remote</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>7 hours ago</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>https://jobright.ai/jobs/info/6aa1f5772f936e4a53daee7c</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>$25/hr - $30/hr</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
         <is>
           <t>RLink Solutions is hiring LLM–AI Quality Analysts for a project evaluating the quality of personalized AI interactions. The role involves designing conversational prompts, assessing AI responses for relevance, grounding, helpfulness, and naturalness, comparing responses, and writing detailed evaluation rationales.
 Responsibilities
@@ -5205,74 +5112,74 @@
 Full-time/Part-time schedule</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
+      <c r="J52" t="inlineStr">
         <is>
           <t>Entry Level</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr">
+      <c r="K52" t="inlineStr">
         <is>
           <t>Full-time, Part-time, Contract</t>
         </is>
       </c>
-      <c r="L53" t="inlineStr">
+      <c r="L52" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr">
+      <c r="M52" t="inlineStr">
         <is>
           <t>2026-09-10 02:12:26</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr">
+      <c r="N52" t="inlineStr">
         <is>
           <t>JobRight</t>
         </is>
       </c>
-      <c r="P53" t="inlineStr">
+      <c r="P52" t="inlineStr">
         <is>
           <t>LinkedIn email 2026-09-10: 'Your application was sent to RLink Solutions' for 'LLM – AI Quality Analyst' (job 4464130549, matches https://www.linkedin.com/jobs/view/4464130549/).</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
+    <row r="53">
+      <c r="A53" t="inlineStr">
         <is>
           <t>greenhouse:twitch:8751076002</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>Software Engineer I, Memberships</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>Twitch</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/twitch/jobs/8751076002?gh_src=Simplify&amp;utm_source=Simplify</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
+      <c r="H53" t="inlineStr">
         <is>
           <t>US, WA, Seattle - Annually $110,500 - $160,000 USD; US, CA, San Francisco - Annually $127,100 - $185,000 USD</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
+      <c r="I53" t="inlineStr">
         <is>
           <t>About Us
 Twitch is the world’s biggest live streaming service, with global communities built around gaming, entertainment, music, sports, cooking, and more. It is where thousands of communities come together for whatever, every day.
@@ -5314,6 +5221,83 @@
 Twitch values your privacy. Please consult our Candidate Privacy Notice, for information about how we collect, use, and disclose personal information of our candidates.</t>
         </is>
       </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>2026-09-10 02:32:03</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Greenhouse</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>Gmail from no-reply@twitchjobs.tv 'Thank you for applying to Twitch' states application has been received. Matches target company Twitch.</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>No Twitch confirmation email in Gmail. Supplied URL page shows Levelpath AI Solutions Specialist success, not Twitch Software Engineer I Memberships, so Twitch submission cannot be confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>url:c2687a3687fbd9e62ec6</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Adobe</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>San Jose</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>https://adobe.wd5.myworkdayjobs.com/en-US/external_experienced/job/San-Jose/Machine-Learning-Engineer_R171645-1/apply/applyManually?jr_id=6a9a209913883870605928bd</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
       <c r="J54" t="inlineStr">
         <is>
           <t>null</t>
@@ -5331,22 +5315,1817 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>2026-09-10 02:32:03</t>
+          <t>2026-09-11 01:36:22</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>Workday</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>Gmail from no-reply@twitchjobs.tv 'Thank you for applying to Twitch' states application has been received. Matches target company Twitch.</t>
-        </is>
-      </c>
-      <c r="Q54" t="inlineStr">
-        <is>
-          <t>No Twitch confirmation email in Gmail. Supplied URL page shows Levelpath AI Solutions Specialist success, not Twitch Software Engineer I Memberships, so Twitch submission cannot be confirmed.</t>
+          <t>Confirmation email from adobe@myworkday.com states received application for R171645 Machine Learning Engineer role, matching Adobe and target title.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>url:160f78d6ee1757ec5a15</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/jobs/info/6aa38b3a626f9945308b1670</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>AI Labs Engineer</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Clasp</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>United States, Remote</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>12 hours ago</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/clasp-group/63dea81e-c456-424a-b88f-446aa2054650/application?utm_source=o5vBVvrWbz&amp;jr_id=6aa38b3a626f9945308b1670</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Clasp is a mission-driven startup expanding access to education and career opportunities through talent solutions and student finance technology. The AI Labs Engineer will help build and improve internal AI tools, owning problems from workflow discovery through product adoption while collaborating with internal users and supporting AI enablement across the company.
+Responsibilities:
+- Own problems from discovery through adoption. Work directly with internal users to understand their workflows, build and launch solutions across the stack, and measure whether they helped
+- Build and improve internal tools. Refine existing agents and create new ones, including their instructions, tools, guardrails, evaluations, and human handoffs
+- Make your work maintainable. Document decisions, setup, risks, and operating steps. Raise architecture, security, privacy, compliance, or production risks early
+- Help Claspmates build with AI. Run programs such as AI Champs, Lattes with AI Labs, and Lunch &amp; Learns, and pair with colleagues to turn ideas into shipped products
+- Keep learning as the field moves. Explore new models, products, and agent patterns, follow what is happening across the industry, and test what is genuinely useful
+Required Qualifications:
+- Evidence you can ship. You have built and shipped at least one tool/product/project beyond your own machine
+- Practical AI fluency. You actively use AI models and development tools. You can explain where they help, where they fail, what you verified yourself, and how you would evaluate quality in a real workflow
+- Full-stack range. You can reason about interfaces, backend logic, APIs and integrations, data flows, testing, and deployment. You do not need equal depth everywhere, but you can own a bounded feature end to end
+- Product judgment. You talk to users, clarify the decision the product should enable, choose the smallest useful version, and measure whether it worked
+- Fast learning. You ask for help with useful context, can operate with incomplete information, want coaching, and apply it
+- If you bring high agency, are ready to dive into unfamiliar problems, and are excited to learn as you go, we want to hear from you
+- To ensure smooth collaboration with the Boston-based team, we are limiting to Eastern/Central timezones with the expectation that it will be Boston hours
+- Additionally, they must be within 1 hour of a medium hub/ large airport with multiple daily flights to Boston
+- We are targeting the broader New England area to start as we expect that the candidate to have frequent travel to Boston for onboarding and ongoing collaboration
+Benefits:
+- Competitive cash and equity compensation.
+- Health benefits, including medical, dental, and vision coverage.
+- Student loan repayment benefits.
+- 401(k) matching.
+- Commuter benefits.
+- Flexible PTO.
+- Opportunities to grow with a fast-moving, mission-driven team.</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Entry Level</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>2026-09-11 03:09:17</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>JobRight</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>Ashby email from Clasp Hiring Team confirms receipt for AI Labs Engineer role at Clasp: 'We've received your application' dated 11 Sep 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>url:74234e98afe7498fb5da</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Gen AI Engineer</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Infosys</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Charlotte, NC</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>3 hours ago</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Infosys is a global digital services and consulting company whose Data and Analytics unit uses advanced AI and analytics to drive business growth and operational efficiency. The Gen AI Engineer will support data preparation, analytics and machine learning model development, validation, deployment, and documentation, while applying generative AI and large language model technologies to translate business needs into actionable solutions.
+Responsibilities
+- Participate in data extraction, transformation, and preparation
+- Resolve common data issues and ensure quality for model development
+- Participate in developing models using statistical or machine learning techniques and collaborate with technology teams to operationalize them into analytics tools or scripts
+- Participate in model testing and validation, selecting the best-performing algorithms based on statistical and business metrics
+- Participate in the development of advanced analytics and machine learning or deep learning models including LLMs using predefined processes and tools like SAS and R/ Python
+- Participate in defining analytics problems; execute visualization, analysis, and predictive modeling with senior support
+- Identify data sources and extract from RDBMS and develop UI/UX for client usage
+- Participate in model performance, while making minor adjustments, and escalate risks or compliance concerns and generate reports on deviations or schedule slippages
+- Proactively participate in detailed documentation of model development, testing, and deployment activities for reproducibility
+- Work closely with business and technology teams to translate requirements into actionable models, while communicating results effectively
+- Apply predefined quality measurement frameworks, if any, to individual project tasks
+- Participate in deploying analytics tools in test and production environment, while ensuring they meet operational requirements
+Qualification
+Generative AI, Large Language Models (LLMs), Agentic Frameworks, Retrieval-Augmented Generation (RAG), Prompt Engineering, Prompt Chaining, Conversational AI, Python, LangChain, LLM Fine-Tuning, Embeddings, Vector Databases, Enterprise Copilots
+Required
+- Experience in Generative AI and Large Language Models (LLMs)
+- Hands-on experience with agentic frameworks (multi-agent systems, tool-using agents, planners)
+- Solid understanding of: RAG architectures, Prompt engineering &amp; prompt chaining, Conversational AI design patterns
+- Bachelor's degree or foreign equivalent required from an accredited institution. Will also consider three years of progressive experience in the specialty in lieu of every year of education
+- This position may require relocation and/or travel to work/project location
+- All applicants authorized to work in the United States are encouraged to apply
+- No H1B
+Preferred
+- Strong programming experience in Python preferred
+- Experience with LangChain / similar orchestration frameworks
+- Exposure to LLM fine-tuning, embeddings, vector databases
+- Experience building enterprise copilots or AI assistants
+- Familiarity with cloud-based GenAI platforms
+Benefits
+- Medical/Dental/Vision/Life Insurance
+- Long-term/Short-term Disability
+- Health and Dependent Care Reimbursement Accounts
+- Insurance (Accident, Critical Illness, Hospital Indemnity, Legal)
+- 401(k) plan and contributions dependent on salary level
+- Paid holidays plus Paid Time Off</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Entry Level</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>2026-09-11 03:32:49</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>Jobright</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>url:b0252476e9b53eb3805f</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/jobs/info/6aa1ef642f936e4a53daebe9</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Software Engineer 1 - IT</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Dell Technologies</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Texas State, Onsite</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>42 minutes ago</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>$90K/yr - $90K/yr</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Dell Technologies is hiring an early-career Software Engineer 1 in its IT Development Program, focused on AI-native software engineering. The role involves rotating across teams to develop AI-powered applications, scalable cloud-native solutions, enterprise integrations, and data-driven technologies while collaborating with cross-functional stakeholders.
+Responsibilities:
+- Develop and deploy AI-powered applications, assistants, agents, and intelligent workflows
+- Build scalable software solutions using cloud-native architectures and modern engineering practices
+- Design and implement integrations across enterprise applications, APIs, data platforms, and AI services
+- Contribute to Retrieval-Augmented Generation (RAG), AI agents, and automation solutions that improve business productivity
+- Partners with architects, product managers, data scientists, and software engineers to deliver end-to-end solutions
+- Apply responsible AI, security, privacy, and governance principles throughout the development lifecycle
+- Participate in CI/CD, monitoring, testing, and operational excellence practices to ensure reliable and scalable solutions
+- Use data and experimentation to improve customer and employee experience
+- Learn emerging technologies quickly and apply them to real-world business challenges
+Required Qualifications:
+- Bachelor's degree in computer science, Computer Engineering, Software Engineering, Artificial Intelligence, or Machine Learning
+- Foundation in software engineering principles, including object-oriented programming, data structures, algorithms, testing, and system design
+- Proficiency in one or more programming languages, such as Python, Java, JavaScript, TypeScript, or C++
+- Hands-on experience developing and deploying AI-powered applications, including work with generative AI, LLMs, AI assistants, agents, prompt engineering, or RAG solutions
+- Demonstrated ability to solve complex problems, communicate effectively, collaborate across teams, and deliver measurable results with accountability
+- Demonstrates curiosity and continuous learning, especially in emerging technologies and AI innovation
+- Takes ownership and accountability for delivering meaningful outcomes
+- Collaborate effectively across teams, disciplines, and geographies
+- Adapts quickly to changing priorities and evolving business needs
+- Uses good judgment and embraces responsibility, ethical technology practices
+- Balances experimentation and innovation with operational excellence
+Preferred:
+- Demonstrated experience developing AI-powered solutions using modern AI/ML frameworks, including assistants, agents, workflow automation, and recommendation systems
+- Knowledge of cloud and software engineering practices, including APIs, microservices, containers, CI/CD, data platforms, and evidence of applied innovation through projects, research, open source, or technical competitions
+Benefits / Program Features:
+- Full-time employment
+- On-site work arrangement
+- Rotational experiences across multiple teams
+- Direct mentorship from technology leaders
+- Opportunities to build innovative solutions
+- Technical expertise, business acumen, leadership capabilities, and a strong network across Dell IT
+Skills: Object-Oriented Programming, Data Structures and Algorithms, Python, Java, JavaScript, TypeScript, C++, Generative AI, Large Language Models (LLMs), AI Agents, Prompt Engineering, Retrieval-Augmented Generation (RAG), Cloud-Native Architecture, APIs, Microservices, Containers, CI/CD</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>New Grad</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>2026-09-11 04:05:40</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>JobRight</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>url:f021dbdd02bbe13a2450</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/jobs/info/6aa39ad5959a10d7230d2b10</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Swarm Aero</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>United States, Remote</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>10 hours ago</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Swarm Aero is redefining air power by building autonomous aircraft and Legion, command and control software for coordinating large numbers of heterogeneous autonomous systems. The Software Engineer Intern will own a scoped project and build, test, integrate, and improve software across frontend, backend, full-stack, real-time, or forward-deployed systems.
+Responsibilities:
+- Build product features across frontend, backend, full-stack, real-time, or forward-deployed software
+- Develop interfaces for telemetry, geospatial data, mission planning, scheduling, collaboration, or system health
+- Build and operate backend services, APIs, event-driven systems, or data pipelines
+- Write automated tests, improve developer tooling, and help ship production-quality software
+- Support integration and test events, debug issues across services and networks, and turn what you learn into product improvements
+Qualification:
+Required:
+- Currently pursuing a degree in Computer Science, Software Engineering, or a closely related field, with graduation and enrollment requirements to be confirmed
+- Strong programming fundamentals and experience building a substantial software project
+- Experience with a modern frontend framework, backend language, systems language, or full-stack application
+- Ability to explain technical tradeoffs, debug methodically, and write maintainable code
+- To conform to U.S. Government export regulations, applicant must be a U.S. citizen, lawful permanent resident of the U.S., protected individual as defined by 8 U.S.C. 1324b(a)(3), or eligible to obtain the required authorizations from the U.S. Department of State
+Preferred:
+- React, TypeScript, Go, Python, Rust, C++, or similar tools
+- Distributed systems, networking, real-time applications, maps, games, simulation, or data visualization
+- Linux, Docker, CI/CD, customer-facing engineering, or deployed project experience
+Skills: React, TypeScript, Go, Python, Rust, C++, Distributed Systems, Real-Time Applications, Linux, Docker, CI/CD
+Benefits:
+- Meaningful equity in a high-growth defense technology company
+- Medical, dental, and vision coverage
+- 401k
+- PTO and paid sick leave
+- Monthly wellness stipend
+- Daily catered lunch (office)
+- Paid parental leave
+- Direct impact on a critical national security mission
+- A world-class team of engineers and operators solving genuinely hard problems
+Company:
+Swarm Aero - Large-scale UAV swarm systems for contested environments.
+Founded in 2022, Oxnard, California, USA, 51-200 employees
+https://www.swarm.aero
+Industries: Aerospace, Artificial Intelligence (AI), Drones, Hardware, National Defense, Military, National Security
+Requirements: No H1B, U.S. Citizen Only</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>New Grad</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>2026-09-11 05:31:57</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>JobRight</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>No qualifying Swarm Aero confirmation email in Gmail. Application page shows Success: Your application was successfully submitted for Software Engineer Intern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>url:daf4a1af49c63d583d60</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/jobs/info/6aa1bb5b0ffb3d4fea6b6b26</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Software Engineer - Early Careers</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Instabase</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>1 day ago</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/swarmaero/04cff1f6-c790-4773-8568-e487a03626f6/application</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Instabase is a people-first company focused on democratizing access to cutting-edge AI innovation and solving unstructured data problems for organizations worldwide. The Software Engineer will design and develop services and applications across the stack, collaborate with cross-functional teams, and contribute to frontend features, platform components, and reusable technologies.
+Responsibilities
+Collaborate with other engineers, product designers, and product managers to drive new features and applications from ideation to implementation to production
+Develop the user interfaces of applications, the core platform, and reusable components
+Evaluating new frontend libraries and technologies to fit our needs and iterating on and maintaining Instabase's frontend stack
+Develop new features that can be leveraged by the other Instabase teams to develop apps and solutions
+Move fast and be empowered to make product and design decisions. You will start contributing to our codebase during your first week, and as an early team member, you will help shape the UI and direction of our product
+Qualification
+Required
+Bachelor's, Master's, or PhD program in Computer Science, Human Computer Interaction, Applied Mathematics, Computer Engineering, or a degree in a related field
+Proficient in one of more of the following languages and frameworks: Python, Go, React, and REST APIs
+Solid communication and collaboration and a strong eagerness to learn
+Preferred
+Preferred graduation date between May 2027 - June 2027
+Benefits
+Flexible PTO: Because life is better when you actually live it!
+Comprehensive Coverage: Top-notch medical, dental, and vision insurance.
+Parental Leave &amp; Fertility Benefits: Supporting you in growing your family, your way.
+Therapy Sessions Covered: Mental health matters—10 free sessions through Samata Health.
+Wellness Stipend: For gym memberships, fitness tech, or whatever keeps you thriving.
+Lunch on Us: Enjoy a lunch credit when you're in the office.</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>New Grad</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>2026-09-11 05:35:47</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>JobRight</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>url:5bb057cb5ae5e6432d31</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/jobs/info/6a739d94e55c73319eb18689</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Software Engineer, New Grad</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Nooks</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>1 hour ago</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/sieve/70847a5f-1262-4163-a496-db4db9fdb138/application?jr_id=6a0ce12b538d03366dc920f0</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>$200K/yr - $200K/yr</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Nooks is an applied AI lab building AI agents and enterprise software for sales and revenue generation. The company is seeking a new graduate software engineer to build full-stack features, develop AI-agent and real-time collaboration systems, work directly with customers, and improve platform performance and scalability.
+Responsibilities
+Design, build, and ship full-stack features using React, TypeScript, Node.js, and Python
+Own projects from initial idea through deployment, monitoring, and iteration
+Work directly with customers to understand problems and turn feedback into product improvements
+Build systems that power AI agents, real-time collaboration, and enterprise-scale workflows
+Improve the performance, reliability, and scalability of our platform
+Write clean, maintainable code and contribute thoughtful code reviews
+Learn from experienced engineers while taking on meaningful ownership from day one
+Qualification - Required
+Are completing or recently completed a Bachelor's or Master's degree in Computer Science or a related technical field
+Have strong computer science fundamentals, including algorithms, data structures, and software design
+Have built software through internships, research, open source, startups, or personal projects
+Love solving difficult technical problems and learning new technologies
+Are excited to work across the stack
+Thrive in fast-moving environments where engineers take ownership and make product decisions
+Enjoy collaborating with teammates and communicating technical ideas clearly
+Can work from our San Francisco office at least three days each week
+Preferred
+Experience with React, TypeScript, Node.js, or Python is a plus, but not required
+Benefits
+Meaningful equity
+Medical insurance
+Dental insurance
+Vision insurance
+Life insurance
+Disability insurance
+Hybrid work
+Unlimited paid time off</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>New Grad</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>2026-09-11 06:57:53</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>JobRight</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>Ashby email from Nooks Hiring Team subject 'We've received your application to Nooks! | Software Engineer, New Grad' confirms receipt for Software Engineer, New Grad at Nooks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>url:d7964e8dbbf8156f1bf2</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/jobs/info/6aa3d951c1928370a285ad24</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Jane Street</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>4 hours ago</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/nooks/311d6e70-5cfa-4e80-89f6-fe00ac1f9f53/application?jr_id=6a739d94e55c73319eb18689</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Software Engineer at Jane Street in New York, NY (Full-time, Onsite, New Grad)
+Jane Street is a financial firm that builds and operates technology systems supporting trading, accounting, research, and infrastructure. The Software Engineer will design and build critical systems and tools, including network monitoring, risk models, data analysis, visualization, and machine learning applications.
+Responsibilities:
+- Design and build the systems and tools that run the firm
+- Solve real problems in critical areas ranging from trading desks to our accounting team
+- Build foundational infrastructure, whether that means implementing network monitoring or risk models
+Qualification:
+- Programming Required
+- A top-notch programmer with a love for technology
+- Intellectually curious, collaborative, and eager to learn
+- Humble and unafraid to ask questions and admit mistakes</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>New Grad</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>2026-09-11 05:53:24</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>Jobright</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>Gmail confirmation from jobs@janestreet.com dated 2026-09-11 subject 'Thank you for applying to Jane Street' stating 'confirm that we received your resume' for Jane Street.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>url:2754cd0d1530549654a3</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/jobs/info/6aa390ab4238ea18d430c992</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Software Engineer, New Grad 2027</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Cursor</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>1 day ago</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Cursor is building tools to automate coding and create the best development experience for professional programmers through research, design, and engineering. The company is hiring new graduate software engineers to own end-to-end product work across user-facing interfaces and underlying systems, including frontend and backend development, prototyping, feature delivery, and product refinement.
+Responsibilities
+- You will design, build, and ship delightful and bulletproof products and systems that engineers love to use every day
+- Adding a small UI improvement so AI-generated code or PRs are easier to read and review
+- Turning a teammate's rough idea into a working prototype over a few days, then iterating based on feedback
+- Shipping a contained feature (frontend + a bit of backend), then fixing bugs and making it feel smoother after people use it
+Qualification
+Required:
+- You're graduating in Spring 2027 (CS, software engineering, computer engineering, or a related technical field)
+- You've already built something great — an app, OSS, or shipped product we can open and review (required)
+- You blend strong engineering and AI tools as leverage without giving up correctness
+- You learn fast, take ownership, and have already done something meaningfully hard early (internships or equivalent industry experience welcome)
+Must-Have Skills: Software Development, Frontend Development, Backend Development, Product Development</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>New Grad</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>2026-09-11 07:13:56</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>JobRight</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>Application was not submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>url:fbbf39159b21d2e320e4</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/jobs/info/6aa39b564233a2201a2b2611</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Software Engineer, New Grad</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Perpay Inc.</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Philadelphia, PA</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>15 hours ago</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/jobs/info/6aa39b564233a2201a2b2611</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Perpay is a mission-driven financial technology company that builds products to improve financial stability and expand access to credit for consumers with subprime credit. The Software Engineer, New Grad will develop, test, and release customer-facing and internal platform features while collaborating with engineering and cross-functional teams. The role also involves writing maintainable code and participating in architecture, design, and code reviews.
+Responsibilities:
+- Develop, test, and release features for our customer-facing and internal platforms alongside the engineering team
+- Write clean, efficient, and maintainable code
+- Collaborate cross-functionally to develop efficient and user-friendly solutions to support the complex needs of our business
+- Actively participate in design reviews, code reviews, and discussions to improve our software architecture and implement efficient processes within our engineering team
+Qualifications:
+- Currently pursuing a Bachelor's degree or higher or a recent graduate studying Computer Science, Mathematics, or a related technical field (or equivalent experience)
+- 1 to 2 previous Software Engineering internships with a focus on fullstack software development
+- Experience with at least one backend application framework such as Django or Flask
+- Experience with frontend technologies such as React, Angular, or Vue.js
+- Knowledge of RESTful API design and integration
+- Experience with Python or another dynamically typed language
+- A strong focus on writing and deploying clear, readable, testable code
+- Ability to pick up new technologies quickly, with software engineering fundamentals being valued more than familiarity with specific tools or languages
+- Eagerness to learn, grow, and seek feedback from team members
+- Strong communication skills
+- This is not a remote opportunity; it is 100% onsite
+Benefits:
+- Equity for full-time team members
+- Premium medical benefits (fully paid base plan, and very reasonable premium for the buy-up option)
+- 5% employer 401k match
+- Unlimited PTO policy
+- Remote weeks around major holidays + extra holiday on weekends like MDW and LDW
+- High quality catered lunch by local chefs, 4 days / week
+- Gym subsidy
+- Paid cell phone + plan
+- Student loan repayment match program
+- Family savings match program
+- Relocation assistance
+- Generous team member discounts
+- Sensible flexibility for personal needs, such as sick children or urgent errands
+- Team events and social gatherings outside of work hours
+- Opportunities to learn and grow alongside other new graduates and experienced engineers</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>New Grad</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>2026-09-11 06:29:26</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>JobRight</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>No qualifying Perpay Gmail confirmation found. Greenhouse confirmation page for perpay token 4034578007 shows 'Thank you for submitting your application!' from The Perpay Hiring Team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>url:31354630cbb53e621dfa</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/jobs/info/6aa1b3b23272060a8e3f19c2</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Software Engineer - New Grad, 2027</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Domino Data Lab</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>United States, Remote</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>1 day ago</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/jobs/info/6aa1b3b23272060a8e3f19c2</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>$150K/yr - $165K/yr</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Domino Data Lab builds software that helps AI-driven organizations develop and operate advanced data science and AI solutions at scale. The New Grad Software Engineer will contribute across the full stack, including backend services, APIs, frontend features, and cloud provider integrations, while working on critical enterprise platform projects.
+Responsibilities:
+As a new grad Software Engineer at Domino, you’ll be working alongside talented engineers from all backgrounds to build the platform that powers how data science is done at some of the world’s largest companies
+Our new grad engineers are versatile and eager to learn, contributing across the full stack - from backend services and APIs, to frontend features, to integrations with cloud providers like AWS, Azure, and GCP
+At Domino, we trust our junior engineers to contribute to critical and high-visibility projects from the start
+You’ll have the opportunity to make a meaningful impact on your team and the company as a whole beginning on day one
+Qualification - Required:
+Strong computer science fundamentals and experience with modern software engineering practices (algorithms, data structures, operating systems, networking, etc.)
+Proficiency with one or more of our core technologies: Python, Go, TypeScript, React, GraphQL, Kubernetes, Docker, Postgres, Redis, Kafka
+Excitement about learning new technologies and contributing to scalable enterprise systems
+Graduating in Spring 2027, currently pursuing a Bachelor's or Master's degree in Computer Science or a related field
+Skills: Algorithms, Data Structures, Operating Systems, Computer Networking, Python, Go, TypeScript, React, GraphQL, Kubernetes, Docker, PostgreSQL, Redis, Apache Kafka
+Benefits:
+This role may be eligible for a sign-on bonus and/or relocation assistance
+Equity
+401(k) plan
+Medical, dental, and vision benefits
+Wellness stipends</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>New Grad</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>2026-09-11 07:04:42</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>JobRight</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>Greenhouse email 'Thank you for applying to Domino' states 'Your application has been received' from Domino.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>url:27261e3eed60193f25a8</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/jobs/info/6a0ce12b538d03366dc920f0</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Member of Technical Staff</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Sieve</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>43 minutes ago</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/embed/job_app?for=dominodatalab&amp;token=7992556&amp;jr_id=6aa1b3b23272060a8e3f19c2</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>$150K/yr - $350K/yr</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Sieve is an AI research lab focused on video data, aiming to solve the bottleneck in the growth of applications powered by high-quality training data. The role involves building and scaling data pipelines, ensuring the delivery of high-quality datasets to customers, and working collaboratively across various teams.
+Responsibilities
+Work across the stack to build and scale the data pipelines that create the datasets we deliver to customers
+Have ownership over projects end-to-end: from how data is sourced and curated, to developing ML filters, improving system efficiency, and building internal dashboards for QA and delivery
+Play a critical role in ensuring customers receive high-quality data on time, every time
+Qualification
+Required
+Strong Python developer, experience in Go or Typescript also welcome
+Excellent communication skills, especially with customers and external teams
+Writes clean, maintainable code
+Able to context switch at a moment's notice
+In-person at our SF HQ
+Preferred
+Experience as an early hire at a startup
+Active GitHub or portfolio projects
+Benefits
+401k + Full Health Insurance
+Breakfast, Lunch, and Dinner covered and your choice of snacks
+Ubers covered home</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Entry Level</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>2026-09-11 06:53:17</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>JobRight</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>No qualifying Sieve Gmail confirmation found. Ashby page for Member of Technical Staff @ Sieve shows 'Success - Your application was successfully submitted.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>url:d5de3ab2c9d3ea29d5c1</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/jobs/info/6a07824e3b54ed42d74cec62</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Makai Labs</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>United States, Remote</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>1 day ago</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>$115K/yr - $130K/yr</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Makai Labs builds software that automates entire companies, and they are seeking an AI Engineer to help build AI systems for enterprise automation. This role involves working closely with engineering and design teams to prototype, ship, and improve AI-powered products and internal tools.
+Industries: Artificial Intelligence (AI), Enterprise Software, Robotics, Software, Robotic Process Automation (RPA)
+Responsibilities
+- Build and improve AI-powered applications and internal tools
+- Rapidly prototype, experiment, and iterate across client and internal projects
+- Implement workflows that use LLMs, retrieval systems, agents, and structured outputs
+- Contribute to shared platform work and reusable tooling
+- Turn prototypes into reliable, client-ready systems
+- Conduct research, benchmarking, testing, and evaluation of new approaches
+- Own smaller projects or sub-projects with guidance from the team
+- Take ownership of deliverables and help deliver work that meets client needs
+- Write and maintain clear internal documentation
+Qualification
+Skills: Python, APIs, Backend services, Workflow automation, FastAPI, Flask, React, TypeScript, Docker, Testing in Python, Testing in TypeScript, Retrieval systems, Embeddings, OCR, Document processing, PDF workflows, Fine-tuning LLMs, Benchmarking LLMs, Serving LLMs, Bias toward action, Willingness to learn quickly
+Required
+- Senior in college, recent graduate, or early-career engineer
+- Background in computer science (bonus if you also have business exposure)
+- Experience building AI applications through internships, coursework, research, or personal projects
+- Experience running AI experiments and iterating quickly
+- Strong Python skills
+Preferred
+- Experience with APIs, backend services, or workflow automation
+- Familiarity with FastAPI, Flask, or similar backend frameworks
+- Familiarity with React and TypeScript
+- Familiarity with Docker and local development environments
+- Familiarity with testing in Python or TypeScript
+- Experience working with retrieval systems, embeddings, or search
+- Experience working with OCR, document processing, or PDF workflows
+- Experience with fine-tuning, benchmarking, or serving LLMs
+- Experience in fast-paced, high-accountability team settings
+Benefits
+- Fully remote role, Eastern time zone
+- Opportunities to work in-person with local colleagues
+- Generous PTO
+- Full health insurance premium reimbursement
+- 401(k) matching
+- Career growth &amp; development opportunities
+Company
+Makai Labs - AI-enabled process automation solutions.
+Founded in 2021
+New York, New York, USA
+11-50 employees
+https://www.makailabs.ai</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>New Grad, Entry Level</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>2026-09-12 01:12:22</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>JobRight</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>Found Ashby confirmation email from Makai Labs Hiring Team confirming application for AI Engineer role at Makai Labs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>url:5f15119907f850137d1d</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/jobs/info/6aa4ee1b2ed333b4ea5c493d</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Jane Street</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>5 minutes ago</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/makai-labs/a350e730-8d80-4528-9d41-497acbd01223/application?jr_id=6a07824e3b54ed42d74cec62</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Software Engineer - New York, NY - Full-time - Onsite - New Grad
+Jane Street is seeking a Software Engineering intern for a hands-on summer internship experience working alongside full-time engineers. The role involves contributing to real-world projects using OCaml and potentially Python, with projects spanning high-performance trading systems, programming language design, and other internal systems.
+Responsibilities:
+- As an intern, you are paired with full-time employees who act as mentors, collaborating with you on real-world projects we actually need done
+- As a Software Engineering intern, you'll learn how we use OCaml (our primary development language) in our day to day work, and gain exposure to the libraries and tools that are foundational to our internal systems
+- Some teams also use Python, so depending on the project, you might do some work with Python as well
+- Mentors design intern projects based on their team's current needs and are heavily invested in helping interns build maintainable, high-quality software that is intended to reach production
+- The projects you will work on are as varied and diverse as those full-timers work on, covering a wide range of problems, from high performance trading systems to programming language design and everything in between
+Qualification:
+- A top-notch programmer with a love for technology
+- Intellectually curious, collaborative, and eager to learn
+- Humble and unafraid to ask questions and admit mistakes
+- Skills Required: Programming, OCaml, Python
+Benefits:
+- A truly unparalleled educational experience
+- Paired with full-time employees who act as mentors
+- Closely mentored by full-time software engineers
+- Intern projects intended to reach production</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>New Grad</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>2026-09-12 01:21:31</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>JobRight</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>Found Jane Street confirmation email from jobs@janestreet.com (2026-09-11) stating 'to confirm that we received your resume' for Software Engineer application.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>url:5c1217f900706fd142b5</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/jobs/info/6a95fedd4c22023a07937681</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Software Engineer, New Grad</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>San Francisco, CA +2 more</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>7 hours ago</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>https://yara.so/jobs/yara-software-engineer-new-grad-552ff909?jr_id=6aa4fa5282e82a31997bb708</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Software Engineer, New Grad - San Francisco, CA (+2 more) - Full-time, Onsite - New Grad
+About the Role:
+Stripe is a technology company building programmable financial infrastructure to help businesses start and scale. The Software Engineer, New Grad will build and deploy software solutions, learn unfamiliar systems, collaborate on coding projects, and contribute to impactful technical initiatives while using AI tools with rigorous judgment.
+Responsibilities:
+- Experience and familiarity with programming, either through side projects or classwork. We work mostly in Java, Ruby, JavaScript, Scala, and Go. We believe new programming languages can be learned if the fundamentals and general knowledge are present
+- Experience from either previous internships or working collaboratively on multi-person coding projects (in a university or professional setting)
+- Ability to learn unfamiliar systems and form an understanding of those systems, through independent research and working with a mentor or subject matter experts
+- Clear written communication skills, with the ability to explain your work to stakeholders, team members, and other Stripes
+- Ability to leverage AI tools to accelerate development while applying rigorous critical thinking and professional judgement to review, refine, and validate all outputs
+- One or more areas of specialized knowledge (frontend, backend, infrastructure or other technologies) balanced with general skills and knowledge
+- Experience in code review practices, and an understanding of how to safely update production systems
+- Familiarity with navigating and managing work in large code bases
+- Experience leading small projects independently, and contributing to larger projects alongside peers
+- Ability to operate with high agency in navigating complex technical obstacles independently, knowing precisely when to unblock oneself and when to ask for help
+Required Qualifications:
+- A Bachelor's or Master's degree in computer science or a directly related field, obtained by summer 2027, or equivalent work experience; New grad candidates should have no more than 18 months of professional experience (excluding internship experience)
+- Experience and familiarity with programming, either through side projects or classwork. We work mostly in Java, Ruby, JavaScript, Scala, and Go. We believe new programming languages can be learned if the fundamentals and general knowledge are present
+- Experience from either previous internships or working collaboratively on multi-person coding projects (in a university or professional setting)
+- Ability to learn unfamiliar systems and form an understanding of those systems, through independent research and working with a mentor or subject matter experts
+- Clear written communication skills, with the ability to explain your work to stakeholders, team members, and other Stripes
+- Ability to leverage AI tools to accelerate development while applying rigorous critical thinking and professional judgement to review, refine, and validate all outputs
+Preferred Qualifications:
+- One or more areas of specialized knowledge (frontend, backend, infrastructure or other technologies) balanced with general skills and knowledge
+- Experience in code review practices, and an understanding of how to safely update production systems
+- Familiarity with navigating and managing work in large code bases
+- Experience leading small projects independently, and contributing to larger projects alongside peers
+- Ability to operate with high agency in navigating complex technical obstacles independently, knowing precisely when to unblock oneself and when to ask for help
+Skills: Programming, Java, Ruby, JavaScript, Scala, Go, Code Review, Large Codebases, AI-Assisted Software Development
+Company: Stripe - Financial services platform for business payments and billing. Founded in 2010. South San Francisco, California, USA. 5001-10000 employees. https://stripe.com</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>New Grad</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>2026-09-12 03:08:40</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>JobRight</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>Greenhouse page shows 'Thank you for applying' and 'Thank you for submitting your application to Stripe.' No qualifying Gmail confirmation email found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>url:797e161607fc662f45e4</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/jobs/info/6a91e328a27a2d3c9848a81e</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Software Engineer Graduate</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Hewlett Packard Enterprise</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Spring, TX</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>7 hours ago</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/Commure/c6a735ef-3d84-4447-94a9-9e8b2dfefced/application?utm_source=PnDq6E4Omw&amp;source=X34Yya61zq&amp;jr_id=6aa47d57f3aa936e2cdb16be</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>$76K/yr - $144K/yr</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Hewlett Packard Enterprise is a global edge-to-cloud company that helps organizations connect, protect, analyze, and act on their data and applications. The Software Engineer Graduate designs, develops, tests, troubleshoots, and debugs software systems while contributing to project teams delivering reliable solutions for low- to moderately-complex products.
+Responsibilities:
+- Codes and programs enhancements, updates, and changes for portions and subsystems of systems software, including operating systems, compliers, networking, utilities, databases, and Internet-related tools
+- Executes established test plans and protocols for assigned portions of code; identifies, logs, and debugs assigned issues
+- Develops understanding of and relationship with internal and outsourced development partners on software systems design and development
+- Participates as a member of a project team of other software systems engineers and internal and outsourced development partners to develop reliable, cost effective and high quality solutions for low to moderately-complex products
+Qualification / Required:
+- Bachelor's or Master's degree in Computer Science, Information Systems, or equivalent
+- Typically, 0-2 years experience
+- Experience or understanding of software systems design tools and languages
+- Good analytical and problem-solving skills
+- Understanding of design for software systems running on multiple platform types
+- Good written and verbal communication skills; mastery in English and local language
+- Understanding of basic testing, coding, and debugging procedures
+Skills: Software Systems Design, Coding, Software Testing, Software Debugging, Cross-Platform Software Development, Written and Verbal Communication
+Benefits:
+- A comprehensive suite of benefits that supports team members' and their loved ones' physical, financial and emotional wellbeing.
+- Specific programs catered to helping employees reach career goals, become knowledge experts, or apply skills to another division.
+- The flexibility to manage work and personal needs.
+- Hybrid work arrangement requiring an average of 2 days per week from an HPE office.
+- Variable incentives may also be offered.</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>New Grad</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>2026-09-12 03:18:54</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>JobRight</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>Page shows 'Application Submitted' dialog stating 'Your application has successfully been submitted' for Software Engineer Graduate. No qualifying Gmail confirmation found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>url:6972c567c589e192e42a</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/jobs/info/6aa495b71d92e2d05d11560e</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Software Engineer, Early Career 2027</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Commure</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Mountain View, CA</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>5 hours ago</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://hpe.wd5.myworkdayjobs.com/en-US/acjobsite/job/Spring%2C-Texas%2C-United-States-of-America/Software-Engineer-Graduate_1213624/apply/applyManually</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>$130K/yr - $150K/yr</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Commure is building an AI-native operating system for healthcare that supports clinical documentation, patient and revenue workflows, and claims processing. The company is seeking early career Software Engineers to build and maintain production features and systems across web, mobile, backend, AI, data, and infrastructure platforms used by healthcare professionals.
+Responsibilities
+- Building product features across our web, mobile, and backend applications, including offline-first experiences for healthcare professionals
+- Developing reliable APIs and backend services that support high-volume clinical workflows
+- Building data processing pipelines for handling complex, high-volume healthcare data
+- Building and improving AI systems: inference pipelines, orchestration (fallbacks, retries, async workflows), and quality evaluation infrastructure
+- Improving monitoring, observability, alerting, debugging, and overall application performance, reliability, and stability
+- Designing internal tools that make engineers faster and production systems easier to operate
+- Working directly with product, design, clinical, and customer-facing teams to understand real-world problems and ship solutions
+Qualification
+Required
+- Bachelor's or Master's degree in Computer Science, Engineering, or a related technical field, graduating recently or within the upcoming academic year
+- Strong fundamentals in algorithms, data structures, operating systems, databases, networking, or distributed systems
+- Experience building software through internships, research, open-source projects, coursework, startups, or personal projects—ideally something substantial outside of coursework
+- Ability to write clean, understandable, and maintainable code
+- Strong debugging and problem-solving skills, especially across multiple layers of a system
+- Curiosity about how complex systems work beyond the component you are directly working on
+- Care about reliability and performance, not just getting a feature to work once
+- High ownership—you care about whether the thing you built actually works for users in production
+- Willingness to learn unfamiliar technologies and move quickly
+- Prefer ownership and autonomy over narrowly scoped tickets
+- Want to work close to users and see the impact of your work quickly
+- Strong communication and ability to work closely with engineers and non-engineers
+Benefits
+- Offers Equity</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>New Grad</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>2026-09-12 02:46:35</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>JobRight</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>url:3407b2be787809763737</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/jobs/info/6aa4fa5282e82a31997bb708</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Software Engineer (New Grad)</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Yara AI</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>United States, Remote</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>57 minutes ago</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Software Engineer (New Grad)
+United States - Full-time - Remote - New Grad
+Yara AI connects new graduate engineers with high-growth companies where they can ship to production immediately and work closely with founders. The role involves owning software surfaces end to end, building with AI tools, and rapidly evaluating the impact of delivered work.
+Computer Software
+Responsibilities
+Ship to production in your first week
+Own a real surface end to end
+Sit near founders and contribute directly
+Build with AI tools daily
+Find out quickly if what you built worked
+Qualification
+TypeScript
+Python
+Go
+GitHub
+Software Deployment
+Software Maintenance
+LLM Application Development
+Required
+• Graduated this year or within the last 18 months
+• Strong GitHub portfolio showcasing your work
+• Built something people have used
+• Experience with TypeScript, Python, or Go
+• Deployed and maintained a project
+• CS degree, bootcamp with real projects, or strong body of work
+• Internships, open-source contributions, or hackathon wins
+• LLM-powered side projects beyond chat wrappers
+• Enthusiasm for work-trial interviews
+• Desire to be an early engineer at a startup
+Benefits
+Ship to production in your first week
+Own a real surface end to end
+Sit near founders and contribute directly
+Build with AI tools daily
+Find out quickly if what you built worked
+Company
+Yara AI
+AI job search agent and personal recruiter.
+San Francisco, California, US
+2-10 employees
+https://www.yara.so/
+Funding Current Stage Early Stage</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>New Grad</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>2026-09-12 03:05:26</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>JobRight</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>Confirmation email from notifications@yara.so confirms receipt of Software Engineer (New Grad) application for Yara Network.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>url:857a446af84d3a4e4646</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/jobs/info/6aa47d57f3aa936e2cdb16be</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Software Engineer, Early Career 2027</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Commure</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Mountain View, CA</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>5 hours ago</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/embed/job_app?for=stripe&amp;jr_id=6a95fedd4c22023a07937681&amp;token=8128744</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>$130K/yr - $150K/yr</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Software Engineer, Early Career 2027 at Commure in Mountain View, CA - Full-time, Onsite
+Compensation: $130K/yr - $150K/yr
+About the Role:
+Commure is building an AI-native operating system for healthcare that supports clinical, administrative, and revenue workflows. The early-career Software Engineer will build and maintain web, mobile, backend, AI, and infrastructure systems used by healthcare professionals, while collaborating with product, design, clinical, and customer-facing teams.
+Industries: Artificial Intelligence (AI), Healthcare, Software, Health Care
+Responsibilities:
+- Building product features across our web, mobile, and backend applications, including offline-first experiences for healthcare professionals
+- Developing reliable APIs and backend services that support high-volume clinical workflows
+- Building data processing pipelines for handling complex, high-volume healthcare data
+- Building and improving AI systems: inference pipelines, orchestration (fallbacks, retries, async workflows), and quality evaluation infrastructure
+- Improving monitoring, observability, alerting, debugging, and overall application performance, reliability, and stability
+- Designing internal tools that make engineers faster and production systems easier to operate
+- Working directly with product, design, clinical, and customer-facing teams to understand real-world problems and ship solutions
+Qualifications:
+Required Skills: Algorithms, Data Structures, Operating Systems, Databases, Computer Networking, Distributed Systems, Software Development, Debugging
+- Bachelor's or Master's degree in Computer Science, Engineering, or a related technical field, graduating recently or within the upcoming academic year
+- Strong fundamentals in algorithms, data structures, operating systems, databases, networking, or distributed systems
+- Experience building software through internships, research, open-source projects, coursework, startups, or personal projects — ideally something substantial outside of coursework
+- Ability to write clean, understandable, and maintainable code
+- Strong debugging and problem-solving skills, especially across multiple layers of a system
+- Curiosity about how complex systems work beyond the component you are directly working on
+- Care about reliability and performance, not just getting a feature to work once
+- High ownership — you care about whether the thing you built actually works for users in production
+- Willingness to learn unfamiliar technologies and move quickly
+- Prefer ownership and autonomy over narrowly scoped tickets
+- Want to work close to users and see the impact of your work quickly
+- Strong communication and ability to work closely with engineers and non-engineers
+About Commure:
+AI-native revenue cycle and ambient documentation platform for health systems.
+Founded in 2017
+Mountain View, California, USA
+1001-5000 employees
+https://commure.com</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>New Grad</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>2026-09-12 03:15:59</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>JobRight</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>Application was not submitted. Automatic recovery exhausted. {"decision": {"is_applied": false, "requires_login": false, "requires_human": false, "human_intervention_reason": "OTHER", "human_intervention_prompt": "Commure application blocked by required transcript upload (Please upload an official or unofficial transcript). No transcript file path was supplied; only the customized resume was provided. Submission verified as not occurred (still on application page with validation error Missing entry for required field). Cannot upload unrelated file per policy."}}</t>
         </is>
       </c>
     </row>

</xml_diff>